<commit_message>
Update Meeting Cadence Doc
</commit_message>
<xml_diff>
--- a/docs/ops/DSAMeetingCadence.xlsx
+++ b/docs/ops/DSAMeetingCadence.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/047a576d2dd5fa45/Desktop/DSA Laboratories/Dev Ops/Meetings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="8_{EBEDAD1E-8C9C-472B-83CB-E1A2ACC0E1F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FD0D8DC-1F3A-4465-8679-E68C19E1CAF6}"/>
+  <xr:revisionPtr revIDLastSave="149" documentId="8_{EBEDAD1E-8C9C-472B-83CB-E1A2ACC0E1F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18AF03C1-5D6C-4CC1-96A8-8961ADAD3D7F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E279F2AC-7B47-4830-8024-308D6F5D13D4}"/>
   </bookViews>
@@ -113,9 +113,6 @@
     <t>Sales / Product Bridge</t>
   </si>
   <si>
-    <t>Every M 11:30PM</t>
-  </si>
-  <si>
     <t>Google Docs</t>
   </si>
   <si>
@@ -126,6 +123,9 @@
   </si>
   <si>
     <t>DSA Leadership</t>
+  </si>
+  <si>
+    <t>Every M 11:30AM</t>
   </si>
 </sst>
 </file>
@@ -1684,7 +1684,7 @@
         <v>12</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>4</v>
@@ -1701,7 +1701,7 @@
         <v>24</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>12</v>
@@ -1710,7 +1710,7 @@
         <v>21</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>9</v>
@@ -1730,7 +1730,7 @@
         <v>12</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>5</v>
@@ -1750,7 +1750,7 @@
         <v>17</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>23</v>

</xml_diff>